<commit_message>
2026.08.29 로직 검증 개선 V2
</commit_message>
<xml_diff>
--- a/output_excel/EL_PA115A02_test_validation.xlsx
+++ b/output_excel/EL_PA115A02_test_validation.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H251"/>
+  <dimension ref="A1:H248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
         <v>-1</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -487,7 +487,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>VAL 자재번호 'EL_PA115A02_1'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 'C11510221G200022'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -506,7 +506,7 @@
         <v>-1</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -515,22 +515,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>VAL 자재번호 'EL_PA115A02_2'가 DB 부품 마스터에 없음</t>
+          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
         <v>-1</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -553,22 +553,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>VAL 자재번호 'EL_PA115A02_3'가 DB 부품 마스터에 없음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         <v>-1</v>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>VAL 자재번호 'C11510221G200022'가 DB 부품 마스터에 없음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>-1</v>
       </c>
       <c r="C9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
         <v>-1</v>
       </c>
       <c r="C10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -810,7 +810,7 @@
         <v>-1</v>
       </c>
       <c r="C11" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -848,7 +848,7 @@
         <v>-1</v>
       </c>
       <c r="C12" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
         <v>-1</v>
       </c>
       <c r="C13" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -924,7 +924,7 @@
         <v>-1</v>
       </c>
       <c r="C14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -981,7 +981,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1000,7 +1000,7 @@
         <v>-1</v>
       </c>
       <c r="C16" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1038,7 +1038,7 @@
         <v>-1</v>
       </c>
       <c r="C17" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1076,7 +1076,7 @@
         <v>-1</v>
       </c>
       <c r="C18" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1114,7 +1114,7 @@
         <v>-1</v>
       </c>
       <c r="C19" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1152,7 +1152,7 @@
         <v>-1</v>
       </c>
       <c r="C20" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1190,7 +1190,7 @@
         <v>-1</v>
       </c>
       <c r="C21" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1228,7 +1228,7 @@
         <v>-1</v>
       </c>
       <c r="C22" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1304,7 +1304,7 @@
         <v>-1</v>
       </c>
       <c r="C24" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>-1</v>
       </c>
       <c r="C25" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1380,7 +1380,7 @@
         <v>-1</v>
       </c>
       <c r="C26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="C27" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1456,7 +1456,7 @@
         <v>-1</v>
       </c>
       <c r="C28" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1494,7 +1494,7 @@
         <v>-1</v>
       </c>
       <c r="C29" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1532,7 +1532,7 @@
         <v>-1</v>
       </c>
       <c r="C30" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1570,7 +1570,7 @@
         <v>-1</v>
       </c>
       <c r="C31" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1608,7 +1608,7 @@
         <v>-1</v>
       </c>
       <c r="C32" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1684,7 +1684,7 @@
         <v>-1</v>
       </c>
       <c r="C34" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1722,7 +1722,7 @@
         <v>-1</v>
       </c>
       <c r="C35" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1760,7 +1760,7 @@
         <v>-1</v>
       </c>
       <c r="C36" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1798,7 +1798,7 @@
         <v>-1</v>
       </c>
       <c r="C37" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1836,7 +1836,7 @@
         <v>-1</v>
       </c>
       <c r="C38" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1874,7 +1874,7 @@
         <v>-1</v>
       </c>
       <c r="C39" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1912,7 +1912,7 @@
         <v>-1</v>
       </c>
       <c r="C40" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1950,7 +1950,7 @@
         <v>-1</v>
       </c>
       <c r="C41" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -1988,7 +1988,7 @@
         <v>-1</v>
       </c>
       <c r="C42" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2026,7 +2026,7 @@
         <v>-1</v>
       </c>
       <c r="C43" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
         <v>-1</v>
       </c>
       <c r="C44" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2102,7 +2102,7 @@
         <v>-1</v>
       </c>
       <c r="C45" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2140,7 +2140,7 @@
         <v>-1</v>
       </c>
       <c r="C46" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         <v>-1</v>
       </c>
       <c r="C47" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2216,7 +2216,7 @@
         <v>-1</v>
       </c>
       <c r="C48" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2254,7 +2254,7 @@
         <v>-1</v>
       </c>
       <c r="C49" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2292,7 +2292,7 @@
         <v>-1</v>
       </c>
       <c r="C50" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2330,7 +2330,7 @@
         <v>-1</v>
       </c>
       <c r="C51" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2368,7 +2368,7 @@
         <v>-1</v>
       </c>
       <c r="C52" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2444,7 +2444,7 @@
         <v>-1</v>
       </c>
       <c r="C54" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         <v>-1</v>
       </c>
       <c r="C55" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2520,7 +2520,7 @@
         <v>-1</v>
       </c>
       <c r="C56" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2558,7 +2558,7 @@
         <v>-1</v>
       </c>
       <c r="C57" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2596,7 +2596,7 @@
         <v>-1</v>
       </c>
       <c r="C58" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2634,7 +2634,7 @@
         <v>-1</v>
       </c>
       <c r="C59" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2672,7 +2672,7 @@
         <v>-1</v>
       </c>
       <c r="C60" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2710,7 +2710,7 @@
         <v>-1</v>
       </c>
       <c r="C61" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2748,7 +2748,7 @@
         <v>-1</v>
       </c>
       <c r="C62" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2833,22 +2833,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>VAL 자재번호 '11500289G07'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -2862,7 +2862,7 @@
         <v>-1</v>
       </c>
       <c r="C65" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2900,7 +2900,7 @@
         <v>-1</v>
       </c>
       <c r="C66" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -2938,7 +2938,7 @@
         <v>-1</v>
       </c>
       <c r="C67" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11500289G07'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 '115C0158G08'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2985,22 +2985,22 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '115C0158G08'가 DB 부품 마스터에 없음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3052,7 +3052,7 @@
         <v>-1</v>
       </c>
       <c r="C70" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3090,7 +3090,7 @@
         <v>-1</v>
       </c>
       <c r="C71" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3109,7 +3109,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3128,7 +3128,7 @@
         <v>-1</v>
       </c>
       <c r="C72" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3185,7 +3185,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3213,22 +3213,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>VAL 자재번호 '115C0158G09'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>-1</v>
       </c>
       <c r="C75" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3251,22 +3251,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '115C0158G09'가 DB 부품 마스터에 없음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
         <v>-1</v>
       </c>
       <c r="C76" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3318,7 +3318,7 @@
         <v>-1</v>
       </c>
       <c r="C77" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3470,7 +3470,7 @@
         <v>-1</v>
       </c>
       <c r="C81" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC1('EL_ATYP')에 CON1 값이 비어있음</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3508,7 +3508,7 @@
         <v>-1</v>
       </c>
       <c r="C82" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3546,7 +3546,7 @@
         <v>-1</v>
       </c>
       <c r="C83" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>SPEC1('EL_ATYP')에 CON1 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -3698,7 +3698,7 @@
         <v>-1</v>
       </c>
       <c r="C87" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3736,7 +3736,7 @@
         <v>-1</v>
       </c>
       <c r="C88" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3774,7 +3774,7 @@
         <v>-1</v>
       </c>
       <c r="C89" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -3812,7 +3812,7 @@
         <v>-1</v>
       </c>
       <c r="C90" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -3850,7 +3850,7 @@
         <v>-1</v>
       </c>
       <c r="C91" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -3888,7 +3888,7 @@
         <v>-1</v>
       </c>
       <c r="C92" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -3926,7 +3926,7 @@
         <v>-1</v>
       </c>
       <c r="C93" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -3964,7 +3964,7 @@
         <v>-1</v>
       </c>
       <c r="C94" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -4002,7 +4002,7 @@
         <v>-1</v>
       </c>
       <c r="C95" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4059,7 +4059,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4078,7 +4078,7 @@
         <v>-1</v>
       </c>
       <c r="C97" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4116,7 +4116,7 @@
         <v>-1</v>
       </c>
       <c r="C98" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4154,7 +4154,7 @@
         <v>-1</v>
       </c>
       <c r="C99" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4192,7 +4192,7 @@
         <v>-1</v>
       </c>
       <c r="C100" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4230,7 +4230,7 @@
         <v>-1</v>
       </c>
       <c r="C101" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -4268,7 +4268,7 @@
         <v>-1</v>
       </c>
       <c r="C102" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4306,7 +4306,7 @@
         <v>-1</v>
       </c>
       <c r="C103" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4344,7 +4344,7 @@
         <v>-1</v>
       </c>
       <c r="C104" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4382,7 +4382,7 @@
         <v>-1</v>
       </c>
       <c r="C105" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -4420,7 +4420,7 @@
         <v>-1</v>
       </c>
       <c r="C106" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -4458,7 +4458,7 @@
         <v>-1</v>
       </c>
       <c r="C107" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -4496,7 +4496,7 @@
         <v>-1</v>
       </c>
       <c r="C108" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4534,7 +4534,7 @@
         <v>-1</v>
       </c>
       <c r="C109" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -4572,7 +4572,7 @@
         <v>-1</v>
       </c>
       <c r="C110" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -4610,7 +4610,7 @@
         <v>-1</v>
       </c>
       <c r="C111" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -4648,7 +4648,7 @@
         <v>-1</v>
       </c>
       <c r="C112" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4686,7 +4686,7 @@
         <v>-1</v>
       </c>
       <c r="C113" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4724,7 +4724,7 @@
         <v>-1</v>
       </c>
       <c r="C114" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4762,7 +4762,7 @@
         <v>-1</v>
       </c>
       <c r="C115" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -4800,7 +4800,7 @@
         <v>-1</v>
       </c>
       <c r="C116" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4819,7 +4819,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -4838,7 +4838,7 @@
         <v>-1</v>
       </c>
       <c r="C117" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4857,7 +4857,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -4876,7 +4876,7 @@
         <v>-1</v>
       </c>
       <c r="C118" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4914,7 +4914,7 @@
         <v>-1</v>
       </c>
       <c r="C119" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4933,7 +4933,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -4952,7 +4952,7 @@
         <v>-1</v>
       </c>
       <c r="C120" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -4990,7 +4990,7 @@
         <v>-1</v>
       </c>
       <c r="C121" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -5104,7 +5104,7 @@
         <v>-1</v>
       </c>
       <c r="C124" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -5142,7 +5142,7 @@
         <v>-1</v>
       </c>
       <c r="C125" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5180,7 +5180,7 @@
         <v>-1</v>
       </c>
       <c r="C126" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5199,7 +5199,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -5332,7 +5332,7 @@
         <v>-1</v>
       </c>
       <c r="C130" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -5370,7 +5370,7 @@
         <v>-1</v>
       </c>
       <c r="C131" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -5389,7 +5389,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -5408,7 +5408,7 @@
         <v>-1</v>
       </c>
       <c r="C132" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -5503,7 +5503,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -5560,7 +5560,7 @@
         <v>-1</v>
       </c>
       <c r="C136" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
         <v>-1</v>
       </c>
       <c r="C137" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -5617,7 +5617,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -5636,7 +5636,7 @@
         <v>-1</v>
       </c>
       <c r="C138" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECGS')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -5788,7 +5788,7 @@
         <v>-1</v>
       </c>
       <c r="C142" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC1('EL_ATYP')에 CON1 값이 비어있음</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -5826,7 +5826,7 @@
         <v>-1</v>
       </c>
       <c r="C143" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC2('EL_ECGV')에 CON2 값이 비어있음</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -5864,7 +5864,7 @@
         <v>-1</v>
       </c>
       <c r="C144" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -5883,7 +5883,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ACD2')에 CON9 값이 비어있음</t>
+          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>SPEC1('EL_ATYP')에 CON1 값이 비어있음</t>
+          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -5997,7 +5997,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>SPEC2('EL_ECGV')에 CON2 값이 비어있음</t>
+          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -6054,7 +6054,7 @@
         <v>-1</v>
       </c>
       <c r="C149" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
+          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -6092,7 +6092,7 @@
         <v>-1</v>
       </c>
       <c r="C150" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -6111,7 +6111,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>SPEC2('EL_ECGV')에 CON2 값이 비어있음</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -6130,7 +6130,7 @@
         <v>-1</v>
       </c>
       <c r="C151" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -6149,7 +6149,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>SPEC7('EL_EHM')에 CON7 값이 비어있음</t>
+          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>SPEC2('EL_ECGV')에 CON2 값이 비어있음</t>
+          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
+          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -6320,7 +6320,7 @@
         <v>-1</v>
       </c>
       <c r="C156" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -6329,22 +6329,22 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ETM')에 CON4 값이 비어있음</t>
+          <t>VAL 자재번호 'V0002633'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -6358,7 +6358,7 @@
         <v>-1</v>
       </c>
       <c r="C157" t="n">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -6367,22 +6367,22 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>SPEC5('EL_EMCBD')에 CON5 값이 비어있음</t>
+          <t>VAL 자재번호 'V0002633'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6396,7 @@
         <v>-1</v>
       </c>
       <c r="C158" t="n">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -6405,22 +6405,22 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECCC')에 CON8 값이 비어있음</t>
+          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -6434,7 +6434,7 @@
         <v>-1</v>
       </c>
       <c r="C159" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -6453,7 +6453,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>VAL 자재번호 'V0002633'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -6472,7 +6472,7 @@
         <v>-1</v>
       </c>
       <c r="C160" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -6491,7 +6491,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>VAL 자재번호 'V0002633'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 '11510132'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -6510,7 +6510,7 @@
         <v>-1</v>
       </c>
       <c r="C161" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 '11510132'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -6548,7 +6548,7 @@
         <v>-1</v>
       </c>
       <c r="C162" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
         <v>-1</v>
       </c>
       <c r="C163" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -6605,7 +6605,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11510132'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -6624,7 +6624,7 @@
         <v>-1</v>
       </c>
       <c r="C164" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -6643,7 +6643,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11510132'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -6662,7 +6662,7 @@
         <v>-1</v>
       </c>
       <c r="C165" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
@@ -6700,7 +6700,7 @@
         <v>-1</v>
       </c>
       <c r="C166" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
@@ -6738,7 +6738,7 @@
         <v>-1</v>
       </c>
       <c r="C167" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
@@ -6776,7 +6776,7 @@
         <v>-1</v>
       </c>
       <c r="C168" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -6795,7 +6795,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
+          <t>VAL 자재번호 '11510023'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -6814,7 +6814,7 @@
         <v>-1</v>
       </c>
       <c r="C169" t="n">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
@@ -6823,22 +6823,22 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
+          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -6852,7 +6852,7 @@
         <v>-1</v>
       </c>
       <c r="C170" t="n">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
@@ -6861,22 +6861,22 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11510162'가 DB 부품 마스터에 없음</t>
+          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -6890,7 +6890,7 @@
         <v>-1</v>
       </c>
       <c r="C171" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
@@ -6899,22 +6899,22 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11510023'가 DB 부품 마스터에 없음</t>
+          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -7042,7 +7042,7 @@
         <v>-1</v>
       </c>
       <c r="C175" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
@@ -7061,7 +7061,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
+          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -7080,7 +7080,7 @@
         <v>-1</v>
       </c>
       <c r="C176" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
@@ -7099,7 +7099,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
+          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
@@ -7118,7 +7118,7 @@
         <v>-1</v>
       </c>
       <c r="C177" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
+          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -7270,7 +7270,7 @@
         <v>-1</v>
       </c>
       <c r="C181" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
@@ -7289,7 +7289,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
+          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -7308,7 +7308,7 @@
         <v>-1</v>
       </c>
       <c r="C182" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
@@ -7327,7 +7327,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
+          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -7346,7 +7346,7 @@
         <v>-1</v>
       </c>
       <c r="C183" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -7403,7 +7403,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
+          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -7469,22 +7469,22 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
+          <t>VAL 자재번호 '11500237'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
         <v>-1</v>
       </c>
       <c r="C187" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
@@ -7517,7 +7517,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
+          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -7536,7 +7536,7 @@
         <v>-1</v>
       </c>
       <c r="C188" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -7574,7 +7574,7 @@
         <v>-1</v>
       </c>
       <c r="C189" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
@@ -7583,22 +7583,22 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11500237'가 DB 부품 마스터에 없음</t>
+          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7631,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -7659,22 +7659,22 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
+          <t>VAL 자재번호 '11500237'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -7707,7 +7707,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
+          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -7726,7 +7726,7 @@
         <v>-1</v>
       </c>
       <c r="C193" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
@@ -7745,7 +7745,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -7764,7 +7764,7 @@
         <v>-1</v>
       </c>
       <c r="C194" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
@@ -7802,7 +7802,7 @@
         <v>-1</v>
       </c>
       <c r="C195" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
@@ -7811,22 +7811,22 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>자재 DB 미존재</t>
+          <t>SPEC만 존재</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>VAL 자재번호 '11500237'가 DB 부품 마스터에 없음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>자재 확인</t>
+          <t>[확인 필요]</t>
         </is>
       </c>
     </row>
@@ -7840,7 +7840,7 @@
         <v>-1</v>
       </c>
       <c r="C196" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
@@ -7878,7 +7878,7 @@
         <v>-1</v>
       </c>
       <c r="C197" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
@@ -7916,7 +7916,7 @@
         <v>-1</v>
       </c>
       <c r="C198" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
@@ -7954,7 +7954,7 @@
         <v>-1</v>
       </c>
       <c r="C199" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
@@ -7992,7 +7992,7 @@
         <v>-1</v>
       </c>
       <c r="C200" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D200" t="inlineStr">
         <is>
@@ -8030,7 +8030,7 @@
         <v>-1</v>
       </c>
       <c r="C201" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D201" t="inlineStr">
         <is>
@@ -8068,7 +8068,7 @@
         <v>-1</v>
       </c>
       <c r="C202" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D202" t="inlineStr">
         <is>
@@ -8106,7 +8106,7 @@
         <v>-1</v>
       </c>
       <c r="C203" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D203" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         <v>-1</v>
       </c>
       <c r="C204" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D204" t="inlineStr">
         <is>
@@ -8182,7 +8182,7 @@
         <v>-1</v>
       </c>
       <c r="C205" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D205" t="inlineStr">
         <is>
@@ -8220,7 +8220,7 @@
         <v>-1</v>
       </c>
       <c r="C206" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
@@ -8258,7 +8258,7 @@
         <v>-1</v>
       </c>
       <c r="C207" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
@@ -8296,7 +8296,7 @@
         <v>-1</v>
       </c>
       <c r="C208" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
@@ -8334,7 +8334,7 @@
         <v>-1</v>
       </c>
       <c r="C209" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D209" t="inlineStr">
         <is>
@@ -8353,7 +8353,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -8372,7 +8372,7 @@
         <v>-1</v>
       </c>
       <c r="C210" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D210" t="inlineStr">
         <is>
@@ -8391,7 +8391,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
+          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -8410,7 +8410,7 @@
         <v>-1</v>
       </c>
       <c r="C211" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D211" t="inlineStr">
         <is>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -8505,7 +8505,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
+          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -8543,7 +8543,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
+          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -8562,7 +8562,7 @@
         <v>-1</v>
       </c>
       <c r="C215" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D215" t="inlineStr">
         <is>
@@ -8600,7 +8600,7 @@
         <v>-1</v>
       </c>
       <c r="C216" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D216" t="inlineStr">
         <is>
@@ -8619,7 +8619,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
+          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -8638,7 +8638,7 @@
         <v>-1</v>
       </c>
       <c r="C217" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D217" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
+          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
+          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -8790,7 +8790,7 @@
         <v>-1</v>
       </c>
       <c r="C221" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D221" t="inlineStr">
         <is>
@@ -8809,7 +8809,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -8828,7 +8828,7 @@
         <v>-1</v>
       </c>
       <c r="C222" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D222" t="inlineStr">
         <is>
@@ -8847,7 +8847,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
+          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -8866,7 +8866,7 @@
         <v>-1</v>
       </c>
       <c r="C223" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D223" t="inlineStr">
         <is>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -8923,7 +8923,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
+          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -8961,7 +8961,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -8980,7 +8980,7 @@
         <v>-1</v>
       </c>
       <c r="C226" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D226" t="inlineStr">
         <is>
@@ -8999,7 +8999,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -9018,7 +9018,7 @@
         <v>-1</v>
       </c>
       <c r="C227" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D227" t="inlineStr">
         <is>
@@ -9037,7 +9037,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -9056,7 +9056,7 @@
         <v>-1</v>
       </c>
       <c r="C228" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D228" t="inlineStr">
         <is>
@@ -9075,7 +9075,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
+          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -9113,7 +9113,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
+          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -9151,7 +9151,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
+          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -9170,7 +9170,7 @@
         <v>-1</v>
       </c>
       <c r="C231" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
@@ -9189,7 +9189,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -9208,7 +9208,7 @@
         <v>-1</v>
       </c>
       <c r="C232" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D232" t="inlineStr">
         <is>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
+          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -9246,7 +9246,7 @@
         <v>-1</v>
       </c>
       <c r="C233" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D233" t="inlineStr">
         <is>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
+          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -9322,7 +9322,7 @@
         <v>-1</v>
       </c>
       <c r="C235" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
@@ -9360,7 +9360,7 @@
         <v>-1</v>
       </c>
       <c r="C236" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
@@ -9379,7 +9379,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -9398,7 +9398,7 @@
         <v>-1</v>
       </c>
       <c r="C237" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
@@ -9417,7 +9417,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
+          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -9455,7 +9455,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -9493,7 +9493,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>SPEC3('EL_AMR')에 CON3 값이 비어있음</t>
+          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -9512,7 +9512,7 @@
         <v>-1</v>
       </c>
       <c r="C240" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D240" t="inlineStr">
         <is>
@@ -9531,7 +9531,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
+          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -9550,7 +9550,7 @@
         <v>-1</v>
       </c>
       <c r="C241" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D241" t="inlineStr">
         <is>
@@ -9569,7 +9569,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>SPEC6('EL_ECWTP')에 CON6 값이 비어있음</t>
+          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -9588,7 +9588,7 @@
         <v>-1</v>
       </c>
       <c r="C242" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -9607,7 +9607,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
+          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -9645,7 +9645,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>SPEC8('EL_ECWSF')에 CON8 값이 비어있음</t>
+          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -9721,7 +9721,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>SPEC5('EL_ECWGP')에 CON5 값이 비어있음</t>
+          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>SPEC4('EL_ECWRL')에 CON4 값이 비어있음</t>
+          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -9778,7 +9778,7 @@
         <v>-1</v>
       </c>
       <c r="C247" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D247" t="inlineStr">
         <is>
@@ -9787,22 +9787,22 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>SPEC7('EL_ETM')에 CON7 값이 비어있음</t>
+          <t>VAL 자재번호 '11510171G01'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>자재 확인</t>
         </is>
       </c>
     </row>
@@ -9816,7 +9816,7 @@
         <v>-1</v>
       </c>
       <c r="C248" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D248" t="inlineStr">
         <is>
@@ -9825,134 +9825,20 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>SPEC만 존재</t>
+          <t>자재 DB 미존재</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>SPEC9('EL_ECWCC')에 CON9 값이 비어있음</t>
+          <t>VAL 자재번호 '11510171G01'가 DB 부품 마스터에 없음</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
-        <is>
-          <t>[확인 필요]</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="inlineStr">
-        <is>
-          <t>EL_PA115A02</t>
-        </is>
-      </c>
-      <c r="B249" t="n">
-        <v>-1</v>
-      </c>
-      <c r="C249" t="n">
-        <v>119</v>
-      </c>
-      <c r="D249" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E249" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="F249" t="inlineStr">
-        <is>
-          <t>SPEC만 존재</t>
-        </is>
-      </c>
-      <c r="G249" t="inlineStr">
-        <is>
-          <t>SPEC10('EL_ACD2')에 CON10 값이 비어있음</t>
-        </is>
-      </c>
-      <c r="H249" t="inlineStr">
-        <is>
-          <t>[확인 필요]</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="inlineStr">
-        <is>
-          <t>EL_PA115A02</t>
-        </is>
-      </c>
-      <c r="B250" t="n">
-        <v>-1</v>
-      </c>
-      <c r="C250" t="n">
-        <v>122</v>
-      </c>
-      <c r="D250" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="F250" t="inlineStr">
-        <is>
-          <t>자재 DB 미존재</t>
-        </is>
-      </c>
-      <c r="G250" t="inlineStr">
-        <is>
-          <t>VAL 자재번호 '11510171G01'가 DB 부품 마스터에 없음</t>
-        </is>
-      </c>
-      <c r="H250" t="inlineStr">
-        <is>
-          <t>자재 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="inlineStr">
-        <is>
-          <t>EL_PA115A02</t>
-        </is>
-      </c>
-      <c r="B251" t="n">
-        <v>-1</v>
-      </c>
-      <c r="C251" t="n">
-        <v>123</v>
-      </c>
-      <c r="D251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="F251" t="inlineStr">
-        <is>
-          <t>자재 DB 미존재</t>
-        </is>
-      </c>
-      <c r="G251" t="inlineStr">
-        <is>
-          <t>VAL 자재번호 '11510171G01'가 DB 부품 마스터에 없음</t>
-        </is>
-      </c>
-      <c r="H251" t="inlineStr">
         <is>
           <t>자재 확인</t>
         </is>

</xml_diff>